<commit_message>
Add specs for drawings 2-6, generator and cross-drawing summary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R9zuNWHVAw4QsHcaJhMbSm
</commit_message>
<xml_diff>
--- a/specs/Wiring_1/Wiring_1_spec.xlsx
+++ b/specs/Wiring_1/Wiring_1_spec.xlsx
@@ -12,15 +12,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Распиновка" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Замечания" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Источники" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Каталог" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Чертёж'!$A$1:$B$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Разъёмы'!$A$1:$P$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Чертёж'!$A$1:$B$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Разъёмы'!$A$1:$M$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Распиновка'!$A$1:$N$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'BOM'!$A$1:$K$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'BOM'!$A$1:$J$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Замечания'!$A$1:$D$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Источники'!$A$1:$B$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Каталог'!$A$1:$H$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -42,7 +42,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -62,11 +62,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8CBAD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -96,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -108,9 +103,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -478,11 +470,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,29 +526,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Исходный файл</t>
+          <t>Лист 1</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Wiring_1_source.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Формат</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>A3, 1 лист, KOMPAS-3D</t>
+          <t>X1 (9-поз.) → кабели 3×0.75 и 4×0.75 (1910 мм) + 2 отвода 1×0.75 (295 мм)  (файл Wiring_1_source.pdf)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B6"/>
+  <autoFilter ref="A1:B5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -567,25 +547,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="34" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -601,34 +578,34 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Обозн.</t>
+          <t>Лист</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Разъём</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Поз. BOM</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Назначение</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>P/N корпуса</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Производитель</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>P/N корпуса</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Тип</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Позиций</t>
@@ -636,35 +613,20 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Занято</t>
+          <t>Контакт (P/N)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Свободно</t>
+          <t>Контактов, шт</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Терминал (P/N)</t>
+          <t>Статус</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Терминалов, шт</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Ответная часть</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Статус</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Примечание</t>
         </is>
@@ -681,20 +643,20 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Основной разъём жгута</t>
-        </is>
+      <c r="E2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>TE Connectivity (AMP)</t>
+          <t>Разъём 9-поз.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -704,41 +666,28 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Корпус 9-поз., 3×3, серия Timer / Micro-Timer II (MCP 1.5), негерметичный, под ножевые контакты 1.6×0.6</t>
+          <t>TE Connectivity</t>
         </is>
       </c>
       <c r="I2" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>964267-2</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>8, 9</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>964267-2</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>928523-1 (по данным DigiKey: mates with 928523) + гнёзда MT II / MCP 1.5</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Подтверждён</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>Ответную часть проверить по чертежу TE (Customer Drawing 928522)</t>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Свободны позиции 8, 9</t>
         </is>
       </c>
     </row>
@@ -753,66 +702,51 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Отводы 295 мм</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Гнёзда FASTON на концах проводов поз.7, 8</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>42238-2</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Концы одиночных проводов поз.7 и поз.8 (295 мм)</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>TE Connectivity (AMP)</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Гнездо FASTON 250 (6.3×0.8), неизолированное, Positive Lock / Fastin-Faston, 0.82–2.08 мм²</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>42238-2</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>Ножевой вывод 6.3×0.8 на ответном устройстве</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Подтверждён</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>0.75 мм² — на нижней границе диапазона, см. замечание 2</t>
-        </is>
-      </c>
+      <c r="M3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -825,69 +759,54 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Концы кабелей</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Наконечники на 7 жилах кабелей поз.5, 6</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Концы жил кабелей поз.5 и поз.6 (7 жил)</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>? (китайская номенклатура DJ…)</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Тип не опознан. Обозначение DJ4xx в китайской номенклатуре обычно — кольцевые/вилочные наконечники</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>DJ451-1</t>
         </is>
       </c>
-      <c r="M4" s="2" t="n">
+      <c r="K4" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Проверить</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>Нужен производитель или фото/эскиз наконечника</t>
-        </is>
-      </c>
+      <c r="M4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P4"/>
+  <autoFilter ref="A1:M4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -902,19 +821,19 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="45" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -930,57 +849,57 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Лист</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Разъём</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>P/N корпуса</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Контакт</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Пин</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Провод №</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Цвет</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Сечение, мм²</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Источник (поз. BOM)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Тип проводника</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Терминал в X1</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Дальний конец</t>
-        </is>
-      </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Терминал на дальнем конце</t>
+          <t>Куда идёт</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Длина, мм</t>
+          <t>Двойной обжим</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Двойной обжим</t>
+          <t>Проверка сечения</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
@@ -1000,48 +919,48 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>928522-1</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>964267-2</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>кабель 6</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>Жёлтый</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Жила кабеля 4×0.75</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>964267-2</t>
-        </is>
-      </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Конец кабеля 6</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>DJ451-1</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>1910</v>
-      </c>
+          <t>Конец кабеля 6 → DJ451-1</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr"/>
     </row>
@@ -1056,174 +975,178 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>928522-1</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>964267-2</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>кабель 6</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Синий</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Жила кабеля 4×0.75</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>964267-2</t>
-        </is>
-      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Конец кабеля 6</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>DJ451-1</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="n">
-        <v>1910</v>
-      </c>
+          <t>Конец кабеля 6 → DJ451-1</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Lada Niva Legend</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>928522-1</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>964267-2</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>поз.7</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Белый</t>
         </is>
       </c>
-      <c r="F4" s="5" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>Одиночный провод 1×0.75</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>964267-2 (общий)</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>Отвод 295 мм</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>42238-2</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="n">
-        <v>295</v>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Отвод 295 мм → 42238-2</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>Пин 3 объединяет белый провод 7 и белую жилу кабеля 5</t>
-        </is>
-      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>1.5 мм² &gt; 1 мм² (макс. 964267-2)</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Lada Niva Legend</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>928522-1</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>964267-2</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>кабель 5</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Белый</t>
         </is>
       </c>
-      <c r="F5" s="5" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Жила кабеля 3×0.75</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>964267-2 (общий)</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Конец кабеля 5</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>DJ451-1</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="n">
-        <v>1910</v>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Конец кабеля 5 → DJ451-1</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr"/>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>1.5 мм² &gt; 1 мм² (макс. 964267-2)</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1236,48 +1159,48 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>928522-1</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>964267-2</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>кабель 5</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Зелёный</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Жила кабеля 3×0.75</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>964267-2</t>
-        </is>
-      </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Конец кабеля 5</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>DJ451-1</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="n">
-        <v>1910</v>
-      </c>
+          <t>Конец кабеля 5 → DJ451-1</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr"/>
     </row>
@@ -1292,48 +1215,48 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>928522-1</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>964267-2</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>поз.8</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Коричневый</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Одиночный провод 1×0.75</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>964267-2</t>
-        </is>
-      </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Отвод 295 мм</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>42238-2</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="n">
-        <v>295</v>
-      </c>
+          <t>Отвод 295 мм → 42238-2</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="inlineStr"/>
     </row>
@@ -1348,174 +1271,186 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>928522-1</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>964267-2</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>кабель 6</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Красный</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Жила кабеля 4×0.75</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>964267-2</t>
-        </is>
-      </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Конец кабеля 6</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>DJ451-1</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="n">
-        <v>1910</v>
-      </c>
+          <t>Конец кабеля 6 → DJ451-1</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="A9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Lada Niva Legend</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>928522-1</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>964267-2</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>кабель 5</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Коричневый</t>
         </is>
       </c>
-      <c r="F9" s="5" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Жила кабеля 3×0.75</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>964267-2 (общий)</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>Конец кабеля 5</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>DJ451-1</t>
-        </is>
-      </c>
-      <c r="L9" s="5" t="n">
-        <v>1910</v>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Конец кабеля 5 → DJ451-1</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
       </c>
-      <c r="N9" s="5" t="inlineStr">
-        <is>
-          <t>Пин 7 объединяет коричневую жилу кабеля 5 и чёрную жилу кабеля 6 (похоже на общий / GND)</t>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>1.5 мм² &gt; 1 мм² (макс. 964267-2)</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Похоже на общий/GND</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Lada Niva Legend</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>928522-1</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>964267-2</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>кабель 6</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Чёрный</t>
         </is>
       </c>
-      <c r="F10" s="5" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>Жила кабеля 4×0.75</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>964267-2 (общий)</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>Конец кабеля 6</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>DJ451-1</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="n">
-        <v>1910</v>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>Конец кабеля 6 → DJ451-1</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
       </c>
-      <c r="N10" s="5" t="inlineStr"/>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>1.5 мм² &gt; 1 мм² (макс. 964267-2)</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>Похоже на общий/GND</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1528,36 +1463,48 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>928522-1</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>964267-2</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Не используется</t>
-        </is>
-      </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>не используется</t>
+        </is>
+      </c>
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Пустая позиция (на виде А перечёркнута)</t>
+          <t>Пустая позиция</t>
         </is>
       </c>
     </row>
@@ -1572,36 +1519,48 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
           <t>X1</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>928522-1</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>964267-2</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Не используется</t>
-        </is>
-      </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>не используется</t>
+        </is>
+      </c>
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Пустая позиция (на виде А перечёркнута)</t>
+          <t>Пустая позиция</t>
         </is>
       </c>
     </row>
@@ -1617,20 +1576,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1646,47 +1604,42 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Лист</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Поз.</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Наименование</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>P/N</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Производитель</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>P/N</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Кол-во</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Ед.</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Где применяется</t>
-        </is>
-      </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Статус</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Примечание</t>
         </is>
       </c>
     </row>
@@ -1699,43 +1652,42 @@
           <t>Lada Niva Legend</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Корпус разъёма 9-поз. (X1)</t>
-        </is>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>Корпус разъёма 9-поз. X1</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>928522-1</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>TE Connectivity</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>928522-1</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>X1</t>
-        </is>
-      </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Подтверждён</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1746,45 +1698,40 @@
           <t>Lada Niva Legend</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Гнездо FASTON 250, неизолир.</t>
-        </is>
-      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>Гнездо FASTON 250</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>42238-2</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>TE Connectivity</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>42238-2</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Концы проводов поз.7, 8</t>
-        </is>
-      </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Подтверждён</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Диапазон 0.82–2.08 мм²</t>
         </is>
       </c>
     </row>
@@ -1797,45 +1744,40 @@
           <t>Lada Niva Legend</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Наконечник</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>DJ451-1</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>?</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>DJ451-1</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="n">
+      <c r="H4" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Концы жил кабелей поз.5, 6</t>
-        </is>
-      </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Проверить</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Тип не опознан</t>
         </is>
       </c>
     </row>
@@ -1848,45 +1790,40 @@
           <t>Lada Niva Legend</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Контакт ножевой 1.6×0.6 (Timer/MT II/MCP 1.5)</t>
-        </is>
-      </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>Контакт ножевой 1.6×0.6</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>964267-2</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
           <t>TE Connectivity</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>964267-2</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="n">
+      <c r="H5" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>X1 пины 1–7</t>
-        </is>
-      </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Подтверждён</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>Диапазон 0.5–1.0 мм², см. замечание 1</t>
         </is>
       </c>
     </row>
@@ -1899,35 +1836,42 @@
           <t>Lada Niva Legend</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Кабель 3×0.75 мм² многопроволочный (белый, зелёный, коричневый)</t>
-        </is>
-      </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>Кабель 3×0.75 мм² (белый, зелёный, коричневый)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="H6" s="2" t="n">
         <v>1.91</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>м</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1938,35 +1882,42 @@
           <t>Lada Niva Legend</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Кабель 4×0.75 мм² многопроволочный (жёлтый, синий, красный, чёрный)</t>
-        </is>
-      </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>Кабель 4×0.75 мм² (жёлтый, синий, красный, чёрный)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="H7" s="2" t="n">
         <v>1.91</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>м</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1977,39 +1928,42 @@
           <t>Lada Niva Legend</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Провод 1×0.75 мм² белый</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="H8" s="2" t="n">
         <v>0.295</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>м</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>X1:3 → FASTON</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -2020,42 +1974,45 @@
           <t>Lada Niva Legend</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Провод 1×0.75 мм² коричневый</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="H9" s="2" t="n">
         <v>0.295</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>м</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>X1:5 → FASTON</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K9"/>
+  <autoFilter ref="A1:J9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2070,9 +2027,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2103,19 +2060,15 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Двойной обжим в X1:3 и X1:7</t>
+          <t>Проверка сечений</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>В пины 3 и 7 заходят по два провода 0.75 мм² (суммарно 1.5 мм²). Диапазон 964267-2 — 0.5–1.0 мм², двойной обжим 2×0.75 в него не входит.</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Вариант А: сращивание (ультразвук или гильза) вне разъёма, в контакт заводить один провод. Вариант Б: контакт той же системы под 1.5–2.5 мм², если корпус его принимает (сверить с чертежом TE). Вариант В: согласовать двойной обжим с TE (application spec).</t>
-        </is>
-      </c>
+          <t>Лист 1, X1, пин 3: двойной обжим поз.7 (белый 0.75) + кабель 5 (белый 0.75) = 1.5 мм² — 1.5 мм² &gt; 1 мм² (макс. 964267-2)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -2123,19 +2076,15 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>FASTON 42238-2 для 0.75 мм²</t>
+          <t>Проверка сечений</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Нижняя граница диапазона 42238-2 — 0.82 мм² (18 AWG). 0.75 мм² — на грани.</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Проверить высоту обжима по application spec TE или взять гнездо FASTON 250 под 0.5–1.0 мм².</t>
-        </is>
-      </c>
+          <t>Лист 1, X1, пин 7: двойной обжим кабель 5 (коричневый 0.75) + кабель 6 (чёрный 0.75) = 1.5 мм² — 1.5 мм² &gt; 1 мм² (макс. 964267-2)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -2143,19 +2092,15 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>DJ451-1</t>
+          <t>Лист 1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Номер в открытых каталогах не найден. Обозначение по китайской номенклатуре (DJ…).</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Уточнить производителя или прислать эскиз (кольцо/вилка, диаметр под винт) — подберу аналог TE/Molex/KST.</t>
-        </is>
-      </c>
+          <t>Размеры: общая длина 1910 мм, отводы поз.7/8 по 295 мм, оболочка кабелей снимается на 95 мм у X1 и на 40 мм на дальнем конце.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -2163,19 +2108,15 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Ответная часть X1</t>
+          <t>Лист 1</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Судя по контактам 964267-2 (нож), 928522-1 — корпус под ножевые контакты; ответный — 928523-1 с гнёздами.</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Если нужна ответная сторона, сверить по Customer Drawing TE.</t>
-        </is>
-      </c>
+          <t>Корпус X1 негерметичный: заглушки на свободные позиции 8, 9 не нужны.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -2183,17 +2124,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Пустые позиции X1:8, X1:9</t>
+          <t>DJ451-1 не опознан</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Корпус негерметичный, заглушки не требуются.</t>
+          <t>Используется во всех чертежах (количество по моделям — в сводке, лист «Потребность по моделям»). В открытых каталогах не найден.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Если в изделии нужна защита от влаги — потребуется другая (герметичная) серия разъёма.</t>
+          <t>Нужен производитель или эскиз.</t>
         </is>
       </c>
     </row>
@@ -2203,17 +2144,17 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Длины</t>
+          <t>Двойной обжим</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Общая длина 1910 мм; отводы поз.7/8 — 295 мм; оболочка кабелей снимается на 95 мм у X1 и на 40 мм на дальнем конце; 50 мм — до конца проводов.</t>
+          <t>Во всех Y-адаптерах основной провод и перемычка обжимаются в один контакт (2×0.75 = 1.5 мм²). Это выше диапазона 964267-2, 927771-3, 927770-1 (до 1.0) и 173645-1/173631-1 (до 1.25).</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Сращивание вне разъёма (ультразвук/гильза) или контакт под 1.5–2.5 мм².</t>
         </is>
       </c>
     </row>
@@ -2229,87 +2170,219 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>P/N</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Серия</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Сечение, мм²</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Аналог / комментарий</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Источник</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>URL</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TE 964267-2</t>
+          <t>928522-1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>https://www.te.com/en/product-964267-2.html</t>
+          <t>TE Connectivity</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Timer / Micro-Timer II</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Корпус 9-поз. 3×3 под ножевые контакты 1.6×0.6, негерметичный</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Подтверждён</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Ответный, по DigiKey, 928523-1</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.digikey.at/en/products/detail/te-connectivity-amp-connectors/928522-1/10461738</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>DigiKey 964267-2</t>
+          <t>964267-2</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>https://www.digikey.com/en/products/detail/te-connectivity-amp-connectors/964267-2/5419549</t>
+          <t>TE Connectivity</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Timer / MT II / MCP 1.5</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Ножевой контакт 1.6×0.6, Sn</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>0.5–1.0</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Подтверждён</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.te.com/en/product-964267-2.html</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>DigiKey 928522-1</t>
+          <t>42238-2</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://www.digikey.at/en/products/detail/te-connectivity-amp-connectors/928522-1/10461738</t>
+          <t>TE Connectivity</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>FASTON 250</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Гнездо 6.3×0.8, неизолированное</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>0.82–2.08</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Подтверждён</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.te.com.cn/chn-zh/product-42238-2.datasheet.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TE 42238-2 datasheet</t>
+          <t>DJ451-1</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>https://www.te.com.cn/chn-zh/product-42238-2.datasheet.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>RS 42238-2</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>https://uk.rs-online.com/web/p/spade-connectors/1709408</t>
-        </is>
-      </c>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>DJ… (китайская номенклатура)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Наконечник, тип по чертежу не определён</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Проверить</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Нужен производитель или эскиз (кольцо/вилка/гильза, диаметр под винт)</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B6"/>
+  <autoFilter ref="A1:H5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>